<commit_message>
Add 96 x 15-minute block schedules for RLDC/SLDC/REMC submission
App: dispatch module gets a D-1 schedule-date picker and CSV/Excel
downloads of the 96-block dispatch (block no, time from/to, MCP,
charge/exchange drawal MW, BTM discharge MW, net MW, interpolated SoC,
action) plus an in-app preview; sizing module gets a 96-block load &
BESS profile download (load, discharge, charge, grid drawal vs contract
demand, ToD window). openpyxl added to requirements for xlsx export.

Excel: new 05_Schedule96 sheet converting the hourly dispatch to 96
blocks by formula (INDEX on hour, TIME-based block boundaries, linear
SoC interpolation, block 96 ending 24:00).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PowerLogic_BESS_Model.xlsx
+++ b/PowerLogic_BESS_Model.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jai_PC\Desktop\BessArbitrageApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D42293E2-87CB-4DEB-897A-64A7447D84BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45B08311-4451-4D50-BA2B-5D501EC3763D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,14 +18,15 @@
     <sheet name="02_Dispatch" sheetId="3" r:id="rId3"/>
     <sheet name="03_Revenue" sheetId="4" r:id="rId4"/>
     <sheet name="04_Container" sheetId="5" r:id="rId5"/>
-    <sheet name="Prices" sheetId="6" r:id="rId6"/>
+    <sheet name="05_Schedule96" sheetId="6" r:id="rId6"/>
+    <sheet name="Prices" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="226">
   <si>
     <t>POWERLOGIC BESS · INDIAN POWER MARKET</t>
   </si>
@@ -658,6 +659,39 @@
   </si>
   <si>
     <t>104S1P — same 5,016 kWh as Design A</t>
+  </si>
+  <si>
+    <t>MODULE 01A · 96-BLOCK SCHEDULE</t>
+  </si>
+  <si>
+    <t>Dispatch converted to 15-minute time blocks — RLDC / SLDC / REMC format</t>
+  </si>
+  <si>
+    <t>Block 1 = 00:00–00:15 … block 96 = 23:45–24:00. Drawal (charging) positive; behind-the-meter discharge is not an injection schedule. Copy into your REMC portal template.</t>
+  </si>
+  <si>
+    <t>Block No</t>
+  </si>
+  <si>
+    <t>Time From</t>
+  </si>
+  <si>
+    <t>Time To</t>
+  </si>
+  <si>
+    <t>Charge / exchange drawal (MW)</t>
+  </si>
+  <si>
+    <t>BTM discharge (MW)</t>
+  </si>
+  <si>
+    <t>Net BESS schedule (MW)</t>
+  </si>
+  <si>
+    <t>SoC end of block (%)</t>
+  </si>
+  <si>
+    <t>SoC is interpolated linearly inside each hour. MW values repeat across the four blocks of an hour — the dispatch plan is hourly; refine block-wise in RTM if needed.</t>
   </si>
   <si>
     <t>Typical day (DAM)</t>
@@ -676,7 +710,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="23">
+  <numFmts count="24">
     <numFmt numFmtId="164" formatCode="#,##0.0&quot; MW&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot; MWh&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0.0&quot; MWh&quot;"/>
@@ -700,6 +734,7 @@
     <numFmt numFmtId="184" formatCode="#,##0.0"/>
     <numFmt numFmtId="185" formatCode="#,##0.000"/>
     <numFmt numFmtId="186" formatCode="#,##0.0&quot; V&quot;"/>
+    <numFmt numFmtId="187" formatCode="0.0"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -803,7 +838,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -891,6 +926,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="187" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5122,6 +5160,3627 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:I103"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="3" width="11" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="39.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="40" t="s">
+        <v>214</v>
+      </c>
+      <c r="B5" s="40" t="s">
+        <v>215</v>
+      </c>
+      <c r="C5" s="40" t="s">
+        <v>216</v>
+      </c>
+      <c r="D5" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="E5" s="40" t="s">
+        <v>217</v>
+      </c>
+      <c r="F5" s="40" t="s">
+        <v>218</v>
+      </c>
+      <c r="G5" s="40" t="s">
+        <v>219</v>
+      </c>
+      <c r="H5" s="40" t="s">
+        <v>220</v>
+      </c>
+      <c r="I5" s="40" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="53">
+        <v>1</v>
+      </c>
+      <c r="B6" s="42" t="str">
+        <f t="shared" ref="B6:B37" si="0">TEXT(TIME(INT((A6-1)*15/60),MOD((A6-1)*15,60),0),"hh:mm")</f>
+        <v>00:00</v>
+      </c>
+      <c r="C6" s="42" t="str">
+        <f t="shared" ref="C6:C37" si="1">IF(A6=96,"24:00",TEXT(TIME(INT(A6*15/60),MOD(A6*15,60),0),"hh:mm"))</f>
+        <v>00:15</v>
+      </c>
+      <c r="D6" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A6-1)/4)+1)</f>
+        <v>4.2</v>
+      </c>
+      <c r="E6" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A6-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A6-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G6" s="45">
+        <f t="shared" ref="G6:G37" si="2">E6-F6</f>
+        <v>0</v>
+      </c>
+      <c r="H6" s="75">
+        <f>100*(IF(INT((A6-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A6-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A6-1)/4)+1)-IF(INT((A6-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A6-1)/4))))*(MOD(A6-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="42" t="str">
+        <f t="shared" ref="I6:I37" si="3">IF(E6&gt;0,"CHARGE",IF(F6&gt;0,"DISCHARGE","—"))</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="53">
+        <v>2</v>
+      </c>
+      <c r="B7" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>00:15</v>
+      </c>
+      <c r="C7" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>00:30</v>
+      </c>
+      <c r="D7" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A7-1)/4)+1)</f>
+        <v>4.2</v>
+      </c>
+      <c r="E7" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A7-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A7-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H7" s="75">
+        <f>100*(IF(INT((A7-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A7-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A7-1)/4)+1)-IF(INT((A7-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A7-1)/4))))*(MOD(A7-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="53">
+        <v>3</v>
+      </c>
+      <c r="B8" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>00:30</v>
+      </c>
+      <c r="C8" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>00:45</v>
+      </c>
+      <c r="D8" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A8-1)/4)+1)</f>
+        <v>4.2</v>
+      </c>
+      <c r="E8" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A8-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A8-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G8" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H8" s="75">
+        <f>100*(IF(INT((A8-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A8-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A8-1)/4)+1)-IF(INT((A8-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A8-1)/4))))*(MOD(A8-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I8" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="53">
+        <v>4</v>
+      </c>
+      <c r="B9" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>00:45</v>
+      </c>
+      <c r="C9" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>01:00</v>
+      </c>
+      <c r="D9" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A9-1)/4)+1)</f>
+        <v>4.2</v>
+      </c>
+      <c r="E9" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A9-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F9" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A9-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G9" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H9" s="75">
+        <f>100*(IF(INT((A9-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A9-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A9-1)/4)+1)-IF(INT((A9-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A9-1)/4))))*(MOD(A9-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="53">
+        <v>5</v>
+      </c>
+      <c r="B10" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>01:00</v>
+      </c>
+      <c r="C10" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>01:15</v>
+      </c>
+      <c r="D10" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A10-1)/4)+1)</f>
+        <v>3.9</v>
+      </c>
+      <c r="E10" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A10-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A10-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H10" s="75">
+        <f>100*(IF(INT((A10-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A10-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A10-1)/4)+1)-IF(INT((A10-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A10-1)/4))))*(MOD(A10-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="53">
+        <v>6</v>
+      </c>
+      <c r="B11" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>01:15</v>
+      </c>
+      <c r="C11" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>01:30</v>
+      </c>
+      <c r="D11" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A11-1)/4)+1)</f>
+        <v>3.9</v>
+      </c>
+      <c r="E11" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A11-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A11-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H11" s="75">
+        <f>100*(IF(INT((A11-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A11-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A11-1)/4)+1)-IF(INT((A11-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A11-1)/4))))*(MOD(A11-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="53">
+        <v>7</v>
+      </c>
+      <c r="B12" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>01:30</v>
+      </c>
+      <c r="C12" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>01:45</v>
+      </c>
+      <c r="D12" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A12-1)/4)+1)</f>
+        <v>3.9</v>
+      </c>
+      <c r="E12" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A12-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A12-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G12" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H12" s="75">
+        <f>100*(IF(INT((A12-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A12-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A12-1)/4)+1)-IF(INT((A12-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A12-1)/4))))*(MOD(A12-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" s="53">
+        <v>8</v>
+      </c>
+      <c r="B13" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>01:45</v>
+      </c>
+      <c r="C13" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>02:00</v>
+      </c>
+      <c r="D13" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A13-1)/4)+1)</f>
+        <v>3.9</v>
+      </c>
+      <c r="E13" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A13-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F13" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A13-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G13" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H13" s="75">
+        <f>100*(IF(INT((A13-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A13-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A13-1)/4)+1)-IF(INT((A13-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A13-1)/4))))*(MOD(A13-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" s="53">
+        <v>9</v>
+      </c>
+      <c r="B14" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>02:00</v>
+      </c>
+      <c r="C14" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>02:15</v>
+      </c>
+      <c r="D14" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A14-1)/4)+1)</f>
+        <v>3.7</v>
+      </c>
+      <c r="E14" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A14-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F14" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A14-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G14" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H14" s="75">
+        <f>100*(IF(INT((A14-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A14-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A14-1)/4)+1)-IF(INT((A14-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A14-1)/4))))*(MOD(A14-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="53">
+        <v>10</v>
+      </c>
+      <c r="B15" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>02:15</v>
+      </c>
+      <c r="C15" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>02:30</v>
+      </c>
+      <c r="D15" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A15-1)/4)+1)</f>
+        <v>3.7</v>
+      </c>
+      <c r="E15" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A15-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A15-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G15" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H15" s="75">
+        <f>100*(IF(INT((A15-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A15-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A15-1)/4)+1)-IF(INT((A15-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A15-1)/4))))*(MOD(A15-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" s="53">
+        <v>11</v>
+      </c>
+      <c r="B16" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>02:30</v>
+      </c>
+      <c r="C16" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>02:45</v>
+      </c>
+      <c r="D16" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A16-1)/4)+1)</f>
+        <v>3.7</v>
+      </c>
+      <c r="E16" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A16-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F16" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A16-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G16" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H16" s="75">
+        <f>100*(IF(INT((A16-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A16-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A16-1)/4)+1)-IF(INT((A16-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A16-1)/4))))*(MOD(A16-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A17" s="53">
+        <v>12</v>
+      </c>
+      <c r="B17" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>02:45</v>
+      </c>
+      <c r="C17" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>03:00</v>
+      </c>
+      <c r="D17" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A17-1)/4)+1)</f>
+        <v>3.7</v>
+      </c>
+      <c r="E17" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A17-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F17" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A17-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G17" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H17" s="75">
+        <f>100*(IF(INT((A17-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A17-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A17-1)/4)+1)-IF(INT((A17-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A17-1)/4))))*(MOD(A17-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I17" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A18" s="53">
+        <v>13</v>
+      </c>
+      <c r="B18" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>03:00</v>
+      </c>
+      <c r="C18" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>03:15</v>
+      </c>
+      <c r="D18" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A18-1)/4)+1)</f>
+        <v>3.6</v>
+      </c>
+      <c r="E18" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A18-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F18" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A18-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G18" s="45">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H18" s="75">
+        <f>100*(IF(INT((A18-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A18-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A18-1)/4)+1)-IF(INT((A18-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A18-1)/4))))*(MOD(A18-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>2.848050967079629</v>
+      </c>
+      <c r="I18" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A19" s="53">
+        <v>14</v>
+      </c>
+      <c r="B19" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>03:15</v>
+      </c>
+      <c r="C19" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>03:30</v>
+      </c>
+      <c r="D19" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A19-1)/4)+1)</f>
+        <v>3.6</v>
+      </c>
+      <c r="E19" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A19-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F19" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A19-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G19" s="45">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H19" s="75">
+        <f>100*(IF(INT((A19-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A19-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A19-1)/4)+1)-IF(INT((A19-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A19-1)/4))))*(MOD(A19-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>5.696101934159258</v>
+      </c>
+      <c r="I19" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A20" s="53">
+        <v>15</v>
+      </c>
+      <c r="B20" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>03:30</v>
+      </c>
+      <c r="C20" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>03:45</v>
+      </c>
+      <c r="D20" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A20-1)/4)+1)</f>
+        <v>3.6</v>
+      </c>
+      <c r="E20" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A20-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F20" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A20-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="45">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H20" s="75">
+        <f>100*(IF(INT((A20-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A20-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A20-1)/4)+1)-IF(INT((A20-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A20-1)/4))))*(MOD(A20-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>8.5441529012388866</v>
+      </c>
+      <c r="I20" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" s="53">
+        <v>16</v>
+      </c>
+      <c r="B21" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>03:45</v>
+      </c>
+      <c r="C21" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>04:00</v>
+      </c>
+      <c r="D21" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A21-1)/4)+1)</f>
+        <v>3.6</v>
+      </c>
+      <c r="E21" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A21-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F21" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A21-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="45">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H21" s="75">
+        <f>100*(IF(INT((A21-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A21-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A21-1)/4)+1)-IF(INT((A21-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A21-1)/4))))*(MOD(A21-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>11.392203868318516</v>
+      </c>
+      <c r="I21" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" s="53">
+        <v>17</v>
+      </c>
+      <c r="B22" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>04:00</v>
+      </c>
+      <c r="C22" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>04:15</v>
+      </c>
+      <c r="D22" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A22-1)/4)+1)</f>
+        <v>3.5</v>
+      </c>
+      <c r="E22" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A22-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F22" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A22-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="45">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H22" s="75">
+        <f>100*(IF(INT((A22-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A22-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A22-1)/4)+1)-IF(INT((A22-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A22-1)/4))))*(MOD(A22-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>14.240254835398144</v>
+      </c>
+      <c r="I22" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" s="53">
+        <v>18</v>
+      </c>
+      <c r="B23" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>04:15</v>
+      </c>
+      <c r="C23" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>04:30</v>
+      </c>
+      <c r="D23" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A23-1)/4)+1)</f>
+        <v>3.5</v>
+      </c>
+      <c r="E23" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A23-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F23" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A23-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="45">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H23" s="75">
+        <f>100*(IF(INT((A23-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A23-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A23-1)/4)+1)-IF(INT((A23-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A23-1)/4))))*(MOD(A23-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>17.088305802477773</v>
+      </c>
+      <c r="I23" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" s="53">
+        <v>19</v>
+      </c>
+      <c r="B24" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>04:30</v>
+      </c>
+      <c r="C24" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>04:45</v>
+      </c>
+      <c r="D24" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A24-1)/4)+1)</f>
+        <v>3.5</v>
+      </c>
+      <c r="E24" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A24-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F24" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A24-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="45">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H24" s="75">
+        <f>100*(IF(INT((A24-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A24-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A24-1)/4)+1)-IF(INT((A24-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A24-1)/4))))*(MOD(A24-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>19.936356769557403</v>
+      </c>
+      <c r="I24" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" s="53">
+        <v>20</v>
+      </c>
+      <c r="B25" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>04:45</v>
+      </c>
+      <c r="C25" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>05:00</v>
+      </c>
+      <c r="D25" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A25-1)/4)+1)</f>
+        <v>3.5</v>
+      </c>
+      <c r="E25" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A25-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F25" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A25-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="45">
+        <f t="shared" si="2"/>
+        <v>8</v>
+      </c>
+      <c r="H25" s="75">
+        <f>100*(IF(INT((A25-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A25-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A25-1)/4)+1)-IF(INT((A25-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A25-1)/4))))*(MOD(A25-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I25" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" s="53">
+        <v>21</v>
+      </c>
+      <c r="B26" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>05:00</v>
+      </c>
+      <c r="C26" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>05:15</v>
+      </c>
+      <c r="D26" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A26-1)/4)+1)</f>
+        <v>3.8</v>
+      </c>
+      <c r="E26" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A26-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A26-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H26" s="75">
+        <f>100*(IF(INT((A26-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A26-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A26-1)/4)+1)-IF(INT((A26-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A26-1)/4))))*(MOD(A26-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I26" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" s="53">
+        <v>22</v>
+      </c>
+      <c r="B27" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>05:15</v>
+      </c>
+      <c r="C27" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>05:30</v>
+      </c>
+      <c r="D27" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A27-1)/4)+1)</f>
+        <v>3.8</v>
+      </c>
+      <c r="E27" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A27-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A27-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H27" s="75">
+        <f>100*(IF(INT((A27-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A27-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A27-1)/4)+1)-IF(INT((A27-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A27-1)/4))))*(MOD(A27-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I27" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28" s="53">
+        <v>23</v>
+      </c>
+      <c r="B28" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>05:30</v>
+      </c>
+      <c r="C28" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>05:45</v>
+      </c>
+      <c r="D28" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A28-1)/4)+1)</f>
+        <v>3.8</v>
+      </c>
+      <c r="E28" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A28-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A28-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H28" s="75">
+        <f>100*(IF(INT((A28-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A28-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A28-1)/4)+1)-IF(INT((A28-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A28-1)/4))))*(MOD(A28-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I28" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29" s="53">
+        <v>24</v>
+      </c>
+      <c r="B29" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>05:45</v>
+      </c>
+      <c r="C29" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>06:00</v>
+      </c>
+      <c r="D29" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A29-1)/4)+1)</f>
+        <v>3.8</v>
+      </c>
+      <c r="E29" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A29-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F29" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A29-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H29" s="75">
+        <f>100*(IF(INT((A29-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A29-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A29-1)/4)+1)-IF(INT((A29-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A29-1)/4))))*(MOD(A29-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I29" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A30" s="53">
+        <v>25</v>
+      </c>
+      <c r="B30" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>06:00</v>
+      </c>
+      <c r="C30" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>06:15</v>
+      </c>
+      <c r="D30" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A30-1)/4)+1)</f>
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="E30" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A30-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F30" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A30-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H30" s="75">
+        <f>100*(IF(INT((A30-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A30-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A30-1)/4)+1)-IF(INT((A30-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A30-1)/4))))*(MOD(A30-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I30" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A31" s="53">
+        <v>26</v>
+      </c>
+      <c r="B31" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>06:15</v>
+      </c>
+      <c r="C31" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>06:30</v>
+      </c>
+      <c r="D31" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A31-1)/4)+1)</f>
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="E31" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A31-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A31-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G31" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H31" s="75">
+        <f>100*(IF(INT((A31-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A31-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A31-1)/4)+1)-IF(INT((A31-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A31-1)/4))))*(MOD(A31-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I31" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A32" s="53">
+        <v>27</v>
+      </c>
+      <c r="B32" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>06:30</v>
+      </c>
+      <c r="C32" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>06:45</v>
+      </c>
+      <c r="D32" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A32-1)/4)+1)</f>
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="E32" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A32-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A32-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H32" s="75">
+        <f>100*(IF(INT((A32-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A32-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A32-1)/4)+1)-IF(INT((A32-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A32-1)/4))))*(MOD(A32-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I32" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A33" s="53">
+        <v>28</v>
+      </c>
+      <c r="B33" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>06:45</v>
+      </c>
+      <c r="C33" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>07:00</v>
+      </c>
+      <c r="D33" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A33-1)/4)+1)</f>
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="E33" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A33-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F33" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A33-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G33" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H33" s="75">
+        <f>100*(IF(INT((A33-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A33-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A33-1)/4)+1)-IF(INT((A33-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A33-1)/4))))*(MOD(A33-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I33" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A34" s="53">
+        <v>29</v>
+      </c>
+      <c r="B34" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>07:00</v>
+      </c>
+      <c r="C34" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>07:15</v>
+      </c>
+      <c r="D34" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A34-1)/4)+1)</f>
+        <v>5.4</v>
+      </c>
+      <c r="E34" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A34-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F34" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A34-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G34" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H34" s="75">
+        <f>100*(IF(INT((A34-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A34-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A34-1)/4)+1)-IF(INT((A34-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A34-1)/4))))*(MOD(A34-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I34" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A35" s="53">
+        <v>30</v>
+      </c>
+      <c r="B35" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>07:15</v>
+      </c>
+      <c r="C35" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>07:30</v>
+      </c>
+      <c r="D35" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A35-1)/4)+1)</f>
+        <v>5.4</v>
+      </c>
+      <c r="E35" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A35-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F35" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A35-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G35" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H35" s="75">
+        <f>100*(IF(INT((A35-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A35-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A35-1)/4)+1)-IF(INT((A35-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A35-1)/4))))*(MOD(A35-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I35" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A36" s="53">
+        <v>31</v>
+      </c>
+      <c r="B36" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>07:30</v>
+      </c>
+      <c r="C36" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>07:45</v>
+      </c>
+      <c r="D36" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A36-1)/4)+1)</f>
+        <v>5.4</v>
+      </c>
+      <c r="E36" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A36-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F36" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A36-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G36" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H36" s="75">
+        <f>100*(IF(INT((A36-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A36-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A36-1)/4)+1)-IF(INT((A36-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A36-1)/4))))*(MOD(A36-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I36" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A37" s="53">
+        <v>32</v>
+      </c>
+      <c r="B37" s="42" t="str">
+        <f t="shared" si="0"/>
+        <v>07:45</v>
+      </c>
+      <c r="C37" s="42" t="str">
+        <f t="shared" si="1"/>
+        <v>08:00</v>
+      </c>
+      <c r="D37" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A37-1)/4)+1)</f>
+        <v>5.4</v>
+      </c>
+      <c r="E37" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A37-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F37" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A37-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H37" s="75">
+        <f>100*(IF(INT((A37-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A37-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A37-1)/4)+1)-IF(INT((A37-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A37-1)/4))))*(MOD(A37-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I37" s="42" t="str">
+        <f t="shared" si="3"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A38" s="53">
+        <v>33</v>
+      </c>
+      <c r="B38" s="42" t="str">
+        <f t="shared" ref="B38:B69" si="4">TEXT(TIME(INT((A38-1)*15/60),MOD((A38-1)*15,60),0),"hh:mm")</f>
+        <v>08:00</v>
+      </c>
+      <c r="C38" s="42" t="str">
+        <f t="shared" ref="C38:C69" si="5">IF(A38=96,"24:00",TEXT(TIME(INT(A38*15/60),MOD(A38*15,60),0),"hh:mm"))</f>
+        <v>08:15</v>
+      </c>
+      <c r="D38" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A38-1)/4)+1)</f>
+        <v>5.2</v>
+      </c>
+      <c r="E38" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A38-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F38" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A38-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G38" s="45">
+        <f t="shared" ref="G38:G69" si="6">E38-F38</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="75">
+        <f>100*(IF(INT((A38-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A38-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A38-1)/4)+1)-IF(INT((A38-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A38-1)/4))))*(MOD(A38-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I38" s="42" t="str">
+        <f t="shared" ref="I38:I69" si="7">IF(E38&gt;0,"CHARGE",IF(F38&gt;0,"DISCHARGE","—"))</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A39" s="53">
+        <v>34</v>
+      </c>
+      <c r="B39" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>08:15</v>
+      </c>
+      <c r="C39" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>08:30</v>
+      </c>
+      <c r="D39" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A39-1)/4)+1)</f>
+        <v>5.2</v>
+      </c>
+      <c r="E39" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A39-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F39" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A39-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G39" s="45">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H39" s="75">
+        <f>100*(IF(INT((A39-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A39-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A39-1)/4)+1)-IF(INT((A39-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A39-1)/4))))*(MOD(A39-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I39" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A40" s="53">
+        <v>35</v>
+      </c>
+      <c r="B40" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>08:30</v>
+      </c>
+      <c r="C40" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>08:45</v>
+      </c>
+      <c r="D40" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A40-1)/4)+1)</f>
+        <v>5.2</v>
+      </c>
+      <c r="E40" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A40-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F40" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A40-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G40" s="45">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H40" s="75">
+        <f>100*(IF(INT((A40-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A40-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A40-1)/4)+1)-IF(INT((A40-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A40-1)/4))))*(MOD(A40-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I40" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A41" s="53">
+        <v>36</v>
+      </c>
+      <c r="B41" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>08:45</v>
+      </c>
+      <c r="C41" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>09:00</v>
+      </c>
+      <c r="D41" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A41-1)/4)+1)</f>
+        <v>5.2</v>
+      </c>
+      <c r="E41" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A41-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F41" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A41-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G41" s="45">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H41" s="75">
+        <f>100*(IF(INT((A41-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A41-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A41-1)/4)+1)-IF(INT((A41-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A41-1)/4))))*(MOD(A41-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I41" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A42" s="53">
+        <v>37</v>
+      </c>
+      <c r="B42" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>09:00</v>
+      </c>
+      <c r="C42" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>09:15</v>
+      </c>
+      <c r="D42" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A42-1)/4)+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E42" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A42-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F42" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A42-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G42" s="45">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H42" s="75">
+        <f>100*(IF(INT((A42-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A42-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A42-1)/4)+1)-IF(INT((A42-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A42-1)/4))))*(MOD(A42-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I42" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A43" s="53">
+        <v>38</v>
+      </c>
+      <c r="B43" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>09:15</v>
+      </c>
+      <c r="C43" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>09:30</v>
+      </c>
+      <c r="D43" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A43-1)/4)+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E43" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A43-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F43" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A43-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G43" s="45">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H43" s="75">
+        <f>100*(IF(INT((A43-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A43-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A43-1)/4)+1)-IF(INT((A43-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A43-1)/4))))*(MOD(A43-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I43" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A44" s="53">
+        <v>39</v>
+      </c>
+      <c r="B44" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>09:30</v>
+      </c>
+      <c r="C44" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>09:45</v>
+      </c>
+      <c r="D44" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A44-1)/4)+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E44" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A44-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F44" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A44-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G44" s="45">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H44" s="75">
+        <f>100*(IF(INT((A44-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A44-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A44-1)/4)+1)-IF(INT((A44-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A44-1)/4))))*(MOD(A44-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I44" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A45" s="53">
+        <v>40</v>
+      </c>
+      <c r="B45" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>09:45</v>
+      </c>
+      <c r="C45" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>10:00</v>
+      </c>
+      <c r="D45" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A45-1)/4)+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E45" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A45-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F45" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A45-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G45" s="45">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H45" s="75">
+        <f>100*(IF(INT((A45-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A45-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A45-1)/4)+1)-IF(INT((A45-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A45-1)/4))))*(MOD(A45-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.784407736637032</v>
+      </c>
+      <c r="I45" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A46" s="53">
+        <v>41</v>
+      </c>
+      <c r="B46" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>10:00</v>
+      </c>
+      <c r="C46" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>10:15</v>
+      </c>
+      <c r="D46" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A46-1)/4)+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E46" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A46-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F46" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A46-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G46" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H46" s="75">
+        <f>100*(IF(INT((A46-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A46-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A46-1)/4)+1)-IF(INT((A46-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A46-1)/4))))*(MOD(A46-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>25.632458703716658</v>
+      </c>
+      <c r="I46" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A47" s="53">
+        <v>42</v>
+      </c>
+      <c r="B47" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>10:15</v>
+      </c>
+      <c r="C47" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>10:30</v>
+      </c>
+      <c r="D47" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A47-1)/4)+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E47" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A47-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F47" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A47-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G47" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H47" s="75">
+        <f>100*(IF(INT((A47-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A47-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A47-1)/4)+1)-IF(INT((A47-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A47-1)/4))))*(MOD(A47-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>28.480509670796287</v>
+      </c>
+      <c r="I47" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A48" s="53">
+        <v>43</v>
+      </c>
+      <c r="B48" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>10:30</v>
+      </c>
+      <c r="C48" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>10:45</v>
+      </c>
+      <c r="D48" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A48-1)/4)+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E48" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A48-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F48" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A48-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G48" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H48" s="75">
+        <f>100*(IF(INT((A48-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A48-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A48-1)/4)+1)-IF(INT((A48-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A48-1)/4))))*(MOD(A48-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>31.328560637875917</v>
+      </c>
+      <c r="I48" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A49" s="53">
+        <v>44</v>
+      </c>
+      <c r="B49" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>10:45</v>
+      </c>
+      <c r="C49" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>11:00</v>
+      </c>
+      <c r="D49" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A49-1)/4)+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E49" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A49-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F49" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A49-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G49" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H49" s="75">
+        <f>100*(IF(INT((A49-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A49-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A49-1)/4)+1)-IF(INT((A49-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A49-1)/4))))*(MOD(A49-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>34.176611604955546</v>
+      </c>
+      <c r="I49" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A50" s="53">
+        <v>45</v>
+      </c>
+      <c r="B50" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>11:00</v>
+      </c>
+      <c r="C50" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>11:15</v>
+      </c>
+      <c r="D50" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A50-1)/4)+1)</f>
+        <v>2.6</v>
+      </c>
+      <c r="E50" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A50-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F50" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A50-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G50" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H50" s="75">
+        <f>100*(IF(INT((A50-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A50-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A50-1)/4)+1)-IF(INT((A50-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A50-1)/4))))*(MOD(A50-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>37.024662572035176</v>
+      </c>
+      <c r="I50" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A51" s="53">
+        <v>46</v>
+      </c>
+      <c r="B51" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>11:15</v>
+      </c>
+      <c r="C51" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>11:30</v>
+      </c>
+      <c r="D51" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A51-1)/4)+1)</f>
+        <v>2.6</v>
+      </c>
+      <c r="E51" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A51-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F51" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A51-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G51" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H51" s="75">
+        <f>100*(IF(INT((A51-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A51-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A51-1)/4)+1)-IF(INT((A51-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A51-1)/4))))*(MOD(A51-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>39.872713539114805</v>
+      </c>
+      <c r="I51" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A52" s="53">
+        <v>47</v>
+      </c>
+      <c r="B52" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>11:30</v>
+      </c>
+      <c r="C52" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>11:45</v>
+      </c>
+      <c r="D52" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A52-1)/4)+1)</f>
+        <v>2.6</v>
+      </c>
+      <c r="E52" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A52-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F52" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A52-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G52" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H52" s="75">
+        <f>100*(IF(INT((A52-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A52-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A52-1)/4)+1)-IF(INT((A52-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A52-1)/4))))*(MOD(A52-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>42.720764506194435</v>
+      </c>
+      <c r="I52" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A53" s="53">
+        <v>48</v>
+      </c>
+      <c r="B53" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>11:45</v>
+      </c>
+      <c r="C53" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>12:00</v>
+      </c>
+      <c r="D53" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A53-1)/4)+1)</f>
+        <v>2.6</v>
+      </c>
+      <c r="E53" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A53-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F53" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A53-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G53" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H53" s="75">
+        <f>100*(IF(INT((A53-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A53-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A53-1)/4)+1)-IF(INT((A53-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A53-1)/4))))*(MOD(A53-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>45.568815473274064</v>
+      </c>
+      <c r="I53" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A54" s="53">
+        <v>49</v>
+      </c>
+      <c r="B54" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>12:00</v>
+      </c>
+      <c r="C54" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>12:15</v>
+      </c>
+      <c r="D54" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A54-1)/4)+1)</f>
+        <v>2.4</v>
+      </c>
+      <c r="E54" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A54-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F54" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A54-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G54" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H54" s="75">
+        <f>100*(IF(INT((A54-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A54-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A54-1)/4)+1)-IF(INT((A54-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A54-1)/4))))*(MOD(A54-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>48.416866440353687</v>
+      </c>
+      <c r="I54" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A55" s="53">
+        <v>50</v>
+      </c>
+      <c r="B55" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>12:15</v>
+      </c>
+      <c r="C55" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>12:30</v>
+      </c>
+      <c r="D55" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A55-1)/4)+1)</f>
+        <v>2.4</v>
+      </c>
+      <c r="E55" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A55-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F55" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A55-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G55" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H55" s="75">
+        <f>100*(IF(INT((A55-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A55-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A55-1)/4)+1)-IF(INT((A55-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A55-1)/4))))*(MOD(A55-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>51.264917407433316</v>
+      </c>
+      <c r="I55" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A56" s="53">
+        <v>51</v>
+      </c>
+      <c r="B56" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>12:30</v>
+      </c>
+      <c r="C56" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>12:45</v>
+      </c>
+      <c r="D56" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A56-1)/4)+1)</f>
+        <v>2.4</v>
+      </c>
+      <c r="E56" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A56-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F56" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A56-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G56" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H56" s="75">
+        <f>100*(IF(INT((A56-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A56-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A56-1)/4)+1)-IF(INT((A56-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A56-1)/4))))*(MOD(A56-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>54.112968374512946</v>
+      </c>
+      <c r="I56" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A57" s="53">
+        <v>52</v>
+      </c>
+      <c r="B57" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>12:45</v>
+      </c>
+      <c r="C57" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>13:00</v>
+      </c>
+      <c r="D57" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A57-1)/4)+1)</f>
+        <v>2.4</v>
+      </c>
+      <c r="E57" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A57-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F57" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A57-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G57" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H57" s="75">
+        <f>100*(IF(INT((A57-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A57-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A57-1)/4)+1)-IF(INT((A57-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A57-1)/4))))*(MOD(A57-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>56.961019341592575</v>
+      </c>
+      <c r="I57" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A58" s="53">
+        <v>53</v>
+      </c>
+      <c r="B58" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>13:00</v>
+      </c>
+      <c r="C58" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>13:15</v>
+      </c>
+      <c r="D58" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A58-1)/4)+1)</f>
+        <v>2.4</v>
+      </c>
+      <c r="E58" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A58-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F58" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A58-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G58" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H58" s="75">
+        <f>100*(IF(INT((A58-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A58-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A58-1)/4)+1)-IF(INT((A58-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A58-1)/4))))*(MOD(A58-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>59.809070308672204</v>
+      </c>
+      <c r="I58" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A59" s="53">
+        <v>54</v>
+      </c>
+      <c r="B59" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>13:15</v>
+      </c>
+      <c r="C59" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>13:30</v>
+      </c>
+      <c r="D59" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A59-1)/4)+1)</f>
+        <v>2.4</v>
+      </c>
+      <c r="E59" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A59-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F59" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A59-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G59" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H59" s="75">
+        <f>100*(IF(INT((A59-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A59-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A59-1)/4)+1)-IF(INT((A59-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A59-1)/4))))*(MOD(A59-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>62.657121275751834</v>
+      </c>
+      <c r="I59" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A60" s="53">
+        <v>55</v>
+      </c>
+      <c r="B60" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>13:30</v>
+      </c>
+      <c r="C60" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>13:45</v>
+      </c>
+      <c r="D60" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A60-1)/4)+1)</f>
+        <v>2.4</v>
+      </c>
+      <c r="E60" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A60-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F60" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A60-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G60" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H60" s="75">
+        <f>100*(IF(INT((A60-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A60-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A60-1)/4)+1)-IF(INT((A60-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A60-1)/4))))*(MOD(A60-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>65.505172242831463</v>
+      </c>
+      <c r="I60" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A61" s="53">
+        <v>56</v>
+      </c>
+      <c r="B61" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>13:45</v>
+      </c>
+      <c r="C61" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>14:00</v>
+      </c>
+      <c r="D61" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A61-1)/4)+1)</f>
+        <v>2.4</v>
+      </c>
+      <c r="E61" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A61-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F61" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A61-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G61" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H61" s="75">
+        <f>100*(IF(INT((A61-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A61-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A61-1)/4)+1)-IF(INT((A61-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A61-1)/4))))*(MOD(A61-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>68.353223209911093</v>
+      </c>
+      <c r="I61" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A62" s="53">
+        <v>57</v>
+      </c>
+      <c r="B62" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>14:00</v>
+      </c>
+      <c r="C62" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>14:15</v>
+      </c>
+      <c r="D62" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A62-1)/4)+1)</f>
+        <v>2.6</v>
+      </c>
+      <c r="E62" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A62-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F62" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A62-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G62" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H62" s="75">
+        <f>100*(IF(INT((A62-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A62-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A62-1)/4)+1)-IF(INT((A62-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A62-1)/4))))*(MOD(A62-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>71.201274176990722</v>
+      </c>
+      <c r="I62" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A63" s="53">
+        <v>58</v>
+      </c>
+      <c r="B63" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>14:15</v>
+      </c>
+      <c r="C63" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>14:30</v>
+      </c>
+      <c r="D63" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A63-1)/4)+1)</f>
+        <v>2.6</v>
+      </c>
+      <c r="E63" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A63-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F63" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A63-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G63" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H63" s="75">
+        <f>100*(IF(INT((A63-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A63-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A63-1)/4)+1)-IF(INT((A63-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A63-1)/4))))*(MOD(A63-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>74.049325144070352</v>
+      </c>
+      <c r="I63" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A64" s="53">
+        <v>59</v>
+      </c>
+      <c r="B64" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>14:30</v>
+      </c>
+      <c r="C64" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>14:45</v>
+      </c>
+      <c r="D64" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A64-1)/4)+1)</f>
+        <v>2.6</v>
+      </c>
+      <c r="E64" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A64-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F64" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A64-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G64" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H64" s="75">
+        <f>100*(IF(INT((A64-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A64-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A64-1)/4)+1)-IF(INT((A64-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A64-1)/4))))*(MOD(A64-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>76.897376111149981</v>
+      </c>
+      <c r="I64" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A65" s="53">
+        <v>60</v>
+      </c>
+      <c r="B65" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>14:45</v>
+      </c>
+      <c r="C65" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>15:00</v>
+      </c>
+      <c r="D65" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A65-1)/4)+1)</f>
+        <v>2.6</v>
+      </c>
+      <c r="E65" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A65-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="F65" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A65-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G65" s="45">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="H65" s="75">
+        <f>100*(IF(INT((A65-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A65-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A65-1)/4)+1)-IF(INT((A65-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A65-1)/4))))*(MOD(A65-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>79.745427078229611</v>
+      </c>
+      <c r="I65" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A66" s="53">
+        <v>61</v>
+      </c>
+      <c r="B66" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>15:00</v>
+      </c>
+      <c r="C66" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>15:15</v>
+      </c>
+      <c r="D66" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A66-1)/4)+1)</f>
+        <v>3.1</v>
+      </c>
+      <c r="E66" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A66-1)/4)+1)</f>
+        <v>7.6363636363636331</v>
+      </c>
+      <c r="F66" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A66-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G66" s="45">
+        <f t="shared" si="6"/>
+        <v>7.6363636363636331</v>
+      </c>
+      <c r="H66" s="75">
+        <f>100*(IF(INT((A66-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A66-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A66-1)/4)+1)-IF(INT((A66-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A66-1)/4))))*(MOD(A66-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>82.464021183169251</v>
+      </c>
+      <c r="I66" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A67" s="53">
+        <v>62</v>
+      </c>
+      <c r="B67" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>15:15</v>
+      </c>
+      <c r="C67" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>15:30</v>
+      </c>
+      <c r="D67" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A67-1)/4)+1)</f>
+        <v>3.1</v>
+      </c>
+      <c r="E67" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A67-1)/4)+1)</f>
+        <v>7.6363636363636331</v>
+      </c>
+      <c r="F67" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A67-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G67" s="45">
+        <f t="shared" si="6"/>
+        <v>7.6363636363636331</v>
+      </c>
+      <c r="H67" s="75">
+        <f>100*(IF(INT((A67-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A67-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A67-1)/4)+1)-IF(INT((A67-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A67-1)/4))))*(MOD(A67-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>85.182615288108892</v>
+      </c>
+      <c r="I67" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A68" s="53">
+        <v>63</v>
+      </c>
+      <c r="B68" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>15:30</v>
+      </c>
+      <c r="C68" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>15:45</v>
+      </c>
+      <c r="D68" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A68-1)/4)+1)</f>
+        <v>3.1</v>
+      </c>
+      <c r="E68" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A68-1)/4)+1)</f>
+        <v>7.6363636363636331</v>
+      </c>
+      <c r="F68" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A68-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G68" s="45">
+        <f t="shared" si="6"/>
+        <v>7.6363636363636331</v>
+      </c>
+      <c r="H68" s="75">
+        <f>100*(IF(INT((A68-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A68-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A68-1)/4)+1)-IF(INT((A68-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A68-1)/4))))*(MOD(A68-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>87.901209393048546</v>
+      </c>
+      <c r="I68" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A69" s="53">
+        <v>64</v>
+      </c>
+      <c r="B69" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>15:45</v>
+      </c>
+      <c r="C69" s="42" t="str">
+        <f t="shared" si="5"/>
+        <v>16:00</v>
+      </c>
+      <c r="D69" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A69-1)/4)+1)</f>
+        <v>3.1</v>
+      </c>
+      <c r="E69" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A69-1)/4)+1)</f>
+        <v>7.6363636363636331</v>
+      </c>
+      <c r="F69" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A69-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G69" s="45">
+        <f t="shared" si="6"/>
+        <v>7.6363636363636331</v>
+      </c>
+      <c r="H69" s="75">
+        <f>100*(IF(INT((A69-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A69-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A69-1)/4)+1)-IF(INT((A69-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A69-1)/4))))*(MOD(A69-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>90.619803497988187</v>
+      </c>
+      <c r="I69" s="42" t="str">
+        <f t="shared" si="7"/>
+        <v>CHARGE</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A70" s="53">
+        <v>65</v>
+      </c>
+      <c r="B70" s="42" t="str">
+        <f t="shared" ref="B70:B101" si="8">TEXT(TIME(INT((A70-1)*15/60),MOD((A70-1)*15,60),0),"hh:mm")</f>
+        <v>16:00</v>
+      </c>
+      <c r="C70" s="42" t="str">
+        <f t="shared" ref="C70:C101" si="9">IF(A70=96,"24:00",TEXT(TIME(INT(A70*15/60),MOD(A70*15,60),0),"hh:mm"))</f>
+        <v>16:15</v>
+      </c>
+      <c r="D70" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A70-1)/4)+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E70" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A70-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F70" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A70-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G70" s="45">
+        <f t="shared" ref="G70:G101" si="10">E70-F70</f>
+        <v>0</v>
+      </c>
+      <c r="H70" s="75">
+        <f>100*(IF(INT((A70-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A70-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A70-1)/4)+1)-IF(INT((A70-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A70-1)/4))))*(MOD(A70-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>90.619803497988187</v>
+      </c>
+      <c r="I70" s="42" t="str">
+        <f t="shared" ref="I70:I101" si="11">IF(E70&gt;0,"CHARGE",IF(F70&gt;0,"DISCHARGE","—"))</f>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A71" s="53">
+        <v>66</v>
+      </c>
+      <c r="B71" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>16:15</v>
+      </c>
+      <c r="C71" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>16:30</v>
+      </c>
+      <c r="D71" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A71-1)/4)+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E71" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A71-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F71" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A71-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G71" s="45">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="H71" s="75">
+        <f>100*(IF(INT((A71-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A71-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A71-1)/4)+1)-IF(INT((A71-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A71-1)/4))))*(MOD(A71-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>90.619803497988187</v>
+      </c>
+      <c r="I71" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A72" s="53">
+        <v>67</v>
+      </c>
+      <c r="B72" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>16:30</v>
+      </c>
+      <c r="C72" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>16:45</v>
+      </c>
+      <c r="D72" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A72-1)/4)+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E72" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A72-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F72" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A72-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G72" s="45">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="H72" s="75">
+        <f>100*(IF(INT((A72-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A72-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A72-1)/4)+1)-IF(INT((A72-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A72-1)/4))))*(MOD(A72-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>90.619803497988187</v>
+      </c>
+      <c r="I72" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A73" s="53">
+        <v>68</v>
+      </c>
+      <c r="B73" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>16:45</v>
+      </c>
+      <c r="C73" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>17:00</v>
+      </c>
+      <c r="D73" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A73-1)/4)+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E73" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A73-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F73" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A73-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="G73" s="45">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="H73" s="75">
+        <f>100*(IF(INT((A73-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A73-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A73-1)/4)+1)-IF(INT((A73-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A73-1)/4))))*(MOD(A73-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>90.619803497988187</v>
+      </c>
+      <c r="I73" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>—</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A74" s="53">
+        <v>69</v>
+      </c>
+      <c r="B74" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>17:00</v>
+      </c>
+      <c r="C74" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>17:15</v>
+      </c>
+      <c r="D74" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A74-1)/4)+1)</f>
+        <v>5.6</v>
+      </c>
+      <c r="E74" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A74-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F74" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A74-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G74" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H74" s="75">
+        <f>100*(IF(INT((A74-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A74-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A74-1)/4)+1)-IF(INT((A74-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A74-1)/4))))*(MOD(A74-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>87.383381944488605</v>
+      </c>
+      <c r="I74" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A75" s="53">
+        <v>70</v>
+      </c>
+      <c r="B75" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>17:15</v>
+      </c>
+      <c r="C75" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>17:30</v>
+      </c>
+      <c r="D75" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A75-1)/4)+1)</f>
+        <v>5.6</v>
+      </c>
+      <c r="E75" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A75-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F75" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A75-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G75" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H75" s="75">
+        <f>100*(IF(INT((A75-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A75-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A75-1)/4)+1)-IF(INT((A75-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A75-1)/4))))*(MOD(A75-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>84.146960390989037</v>
+      </c>
+      <c r="I75" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A76" s="53">
+        <v>71</v>
+      </c>
+      <c r="B76" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>17:30</v>
+      </c>
+      <c r="C76" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>17:45</v>
+      </c>
+      <c r="D76" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A76-1)/4)+1)</f>
+        <v>5.6</v>
+      </c>
+      <c r="E76" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A76-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F76" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A76-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G76" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H76" s="75">
+        <f>100*(IF(INT((A76-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A76-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A76-1)/4)+1)-IF(INT((A76-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A76-1)/4))))*(MOD(A76-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>80.91053883748944</v>
+      </c>
+      <c r="I76" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A77" s="53">
+        <v>72</v>
+      </c>
+      <c r="B77" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>17:45</v>
+      </c>
+      <c r="C77" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>18:00</v>
+      </c>
+      <c r="D77" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A77-1)/4)+1)</f>
+        <v>5.6</v>
+      </c>
+      <c r="E77" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A77-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F77" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A77-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G77" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H77" s="75">
+        <f>100*(IF(INT((A77-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A77-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A77-1)/4)+1)-IF(INT((A77-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A77-1)/4))))*(MOD(A77-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>77.674117283989872</v>
+      </c>
+      <c r="I77" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A78" s="53">
+        <v>73</v>
+      </c>
+      <c r="B78" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>18:00</v>
+      </c>
+      <c r="C78" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>18:15</v>
+      </c>
+      <c r="D78" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A78-1)/4)+1)</f>
+        <v>7.2</v>
+      </c>
+      <c r="E78" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A78-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A78-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G78" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H78" s="75">
+        <f>100*(IF(INT((A78-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A78-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A78-1)/4)+1)-IF(INT((A78-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A78-1)/4))))*(MOD(A78-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>74.43769573049029</v>
+      </c>
+      <c r="I78" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A79" s="53">
+        <v>74</v>
+      </c>
+      <c r="B79" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>18:15</v>
+      </c>
+      <c r="C79" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>18:30</v>
+      </c>
+      <c r="D79" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A79-1)/4)+1)</f>
+        <v>7.2</v>
+      </c>
+      <c r="E79" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A79-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F79" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A79-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G79" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H79" s="75">
+        <f>100*(IF(INT((A79-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A79-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A79-1)/4)+1)-IF(INT((A79-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A79-1)/4))))*(MOD(A79-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>71.201274176990708</v>
+      </c>
+      <c r="I79" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A80" s="53">
+        <v>75</v>
+      </c>
+      <c r="B80" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>18:30</v>
+      </c>
+      <c r="C80" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>18:45</v>
+      </c>
+      <c r="D80" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A80-1)/4)+1)</f>
+        <v>7.2</v>
+      </c>
+      <c r="E80" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A80-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F80" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A80-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G80" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H80" s="75">
+        <f>100*(IF(INT((A80-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A80-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A80-1)/4)+1)-IF(INT((A80-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A80-1)/4))))*(MOD(A80-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>67.964852623491126</v>
+      </c>
+      <c r="I80" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A81" s="53">
+        <v>76</v>
+      </c>
+      <c r="B81" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>18:45</v>
+      </c>
+      <c r="C81" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>19:00</v>
+      </c>
+      <c r="D81" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A81-1)/4)+1)</f>
+        <v>7.2</v>
+      </c>
+      <c r="E81" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A81-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F81" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A81-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G81" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H81" s="75">
+        <f>100*(IF(INT((A81-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A81-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A81-1)/4)+1)-IF(INT((A81-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A81-1)/4))))*(MOD(A81-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>64.728431069991558</v>
+      </c>
+      <c r="I81" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A82" s="53">
+        <v>77</v>
+      </c>
+      <c r="B82" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>19:00</v>
+      </c>
+      <c r="C82" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>19:15</v>
+      </c>
+      <c r="D82" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A82-1)/4)+1)</f>
+        <v>8.5</v>
+      </c>
+      <c r="E82" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A82-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F82" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A82-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G82" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H82" s="75">
+        <f>100*(IF(INT((A82-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A82-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A82-1)/4)+1)-IF(INT((A82-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A82-1)/4))))*(MOD(A82-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>61.492009516491969</v>
+      </c>
+      <c r="I82" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A83" s="53">
+        <v>78</v>
+      </c>
+      <c r="B83" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>19:15</v>
+      </c>
+      <c r="C83" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>19:30</v>
+      </c>
+      <c r="D83" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A83-1)/4)+1)</f>
+        <v>8.5</v>
+      </c>
+      <c r="E83" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A83-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F83" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A83-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G83" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H83" s="75">
+        <f>100*(IF(INT((A83-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A83-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A83-1)/4)+1)-IF(INT((A83-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A83-1)/4))))*(MOD(A83-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>58.255587962992394</v>
+      </c>
+      <c r="I83" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A84" s="53">
+        <v>79</v>
+      </c>
+      <c r="B84" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>19:30</v>
+      </c>
+      <c r="C84" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>19:45</v>
+      </c>
+      <c r="D84" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A84-1)/4)+1)</f>
+        <v>8.5</v>
+      </c>
+      <c r="E84" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A84-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F84" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A84-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G84" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H84" s="75">
+        <f>100*(IF(INT((A84-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A84-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A84-1)/4)+1)-IF(INT((A84-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A84-1)/4))))*(MOD(A84-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>55.019166409492811</v>
+      </c>
+      <c r="I84" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A85" s="53">
+        <v>80</v>
+      </c>
+      <c r="B85" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>19:45</v>
+      </c>
+      <c r="C85" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>20:00</v>
+      </c>
+      <c r="D85" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A85-1)/4)+1)</f>
+        <v>8.5</v>
+      </c>
+      <c r="E85" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A85-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F85" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A85-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G85" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H85" s="75">
+        <f>100*(IF(INT((A85-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A85-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A85-1)/4)+1)-IF(INT((A85-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A85-1)/4))))*(MOD(A85-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>51.782744855993236</v>
+      </c>
+      <c r="I85" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A86" s="53">
+        <v>81</v>
+      </c>
+      <c r="B86" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>20:00</v>
+      </c>
+      <c r="C86" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>20:15</v>
+      </c>
+      <c r="D86" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A86-1)/4)+1)</f>
+        <v>8.9</v>
+      </c>
+      <c r="E86" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A86-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F86" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A86-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G86" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H86" s="75">
+        <f>100*(IF(INT((A86-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A86-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A86-1)/4)+1)-IF(INT((A86-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A86-1)/4))))*(MOD(A86-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>48.546323302493661</v>
+      </c>
+      <c r="I86" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A87" s="53">
+        <v>82</v>
+      </c>
+      <c r="B87" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>20:15</v>
+      </c>
+      <c r="C87" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>20:30</v>
+      </c>
+      <c r="D87" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A87-1)/4)+1)</f>
+        <v>8.9</v>
+      </c>
+      <c r="E87" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A87-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F87" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A87-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G87" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H87" s="75">
+        <f>100*(IF(INT((A87-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A87-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A87-1)/4)+1)-IF(INT((A87-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A87-1)/4))))*(MOD(A87-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>45.309901748994079</v>
+      </c>
+      <c r="I87" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A88" s="53">
+        <v>83</v>
+      </c>
+      <c r="B88" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>20:30</v>
+      </c>
+      <c r="C88" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>20:45</v>
+      </c>
+      <c r="D88" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A88-1)/4)+1)</f>
+        <v>8.9</v>
+      </c>
+      <c r="E88" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A88-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F88" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A88-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G88" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H88" s="75">
+        <f>100*(IF(INT((A88-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A88-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A88-1)/4)+1)-IF(INT((A88-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A88-1)/4))))*(MOD(A88-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>42.073480195494497</v>
+      </c>
+      <c r="I88" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A89" s="53">
+        <v>84</v>
+      </c>
+      <c r="B89" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>20:45</v>
+      </c>
+      <c r="C89" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>21:00</v>
+      </c>
+      <c r="D89" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A89-1)/4)+1)</f>
+        <v>8.9</v>
+      </c>
+      <c r="E89" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A89-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F89" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A89-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G89" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H89" s="75">
+        <f>100*(IF(INT((A89-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A89-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A89-1)/4)+1)-IF(INT((A89-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A89-1)/4))))*(MOD(A89-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>38.837058641994922</v>
+      </c>
+      <c r="I89" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A90" s="53">
+        <v>85</v>
+      </c>
+      <c r="B90" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>21:00</v>
+      </c>
+      <c r="C90" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>21:15</v>
+      </c>
+      <c r="D90" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A90-1)/4)+1)</f>
+        <v>7.8</v>
+      </c>
+      <c r="E90" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A90-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F90" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A90-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G90" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H90" s="75">
+        <f>100*(IF(INT((A90-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A90-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A90-1)/4)+1)-IF(INT((A90-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A90-1)/4))))*(MOD(A90-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>35.60063708849534</v>
+      </c>
+      <c r="I90" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A91" s="53">
+        <v>86</v>
+      </c>
+      <c r="B91" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>21:15</v>
+      </c>
+      <c r="C91" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>21:30</v>
+      </c>
+      <c r="D91" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A91-1)/4)+1)</f>
+        <v>7.8</v>
+      </c>
+      <c r="E91" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A91-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F91" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A91-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G91" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H91" s="75">
+        <f>100*(IF(INT((A91-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A91-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A91-1)/4)+1)-IF(INT((A91-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A91-1)/4))))*(MOD(A91-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>32.364215534995758</v>
+      </c>
+      <c r="I91" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A92" s="53">
+        <v>87</v>
+      </c>
+      <c r="B92" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>21:30</v>
+      </c>
+      <c r="C92" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>21:45</v>
+      </c>
+      <c r="D92" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A92-1)/4)+1)</f>
+        <v>7.8</v>
+      </c>
+      <c r="E92" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A92-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F92" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A92-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G92" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H92" s="75">
+        <f>100*(IF(INT((A92-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A92-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A92-1)/4)+1)-IF(INT((A92-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A92-1)/4))))*(MOD(A92-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>29.127793981496183</v>
+      </c>
+      <c r="I92" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A93" s="53">
+        <v>88</v>
+      </c>
+      <c r="B93" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>21:45</v>
+      </c>
+      <c r="C93" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>22:00</v>
+      </c>
+      <c r="D93" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A93-1)/4)+1)</f>
+        <v>7.8</v>
+      </c>
+      <c r="E93" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A93-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F93" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A93-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G93" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H93" s="75">
+        <f>100*(IF(INT((A93-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A93-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A93-1)/4)+1)-IF(INT((A93-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A93-1)/4))))*(MOD(A93-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>25.891372427996604</v>
+      </c>
+      <c r="I93" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A94" s="53">
+        <v>89</v>
+      </c>
+      <c r="B94" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>22:00</v>
+      </c>
+      <c r="C94" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>22:15</v>
+      </c>
+      <c r="D94" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A94-1)/4)+1)</f>
+        <v>6.2</v>
+      </c>
+      <c r="E94" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A94-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F94" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A94-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G94" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H94" s="75">
+        <f>100*(IF(INT((A94-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A94-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A94-1)/4)+1)-IF(INT((A94-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A94-1)/4))))*(MOD(A94-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>22.654950874497022</v>
+      </c>
+      <c r="I94" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A95" s="53">
+        <v>90</v>
+      </c>
+      <c r="B95" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>22:15</v>
+      </c>
+      <c r="C95" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>22:30</v>
+      </c>
+      <c r="D95" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A95-1)/4)+1)</f>
+        <v>6.2</v>
+      </c>
+      <c r="E95" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A95-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F95" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A95-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G95" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H95" s="75">
+        <f>100*(IF(INT((A95-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A95-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A95-1)/4)+1)-IF(INT((A95-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A95-1)/4))))*(MOD(A95-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>19.418529320997443</v>
+      </c>
+      <c r="I95" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A96" s="53">
+        <v>91</v>
+      </c>
+      <c r="B96" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>22:30</v>
+      </c>
+      <c r="C96" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>22:45</v>
+      </c>
+      <c r="D96" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A96-1)/4)+1)</f>
+        <v>6.2</v>
+      </c>
+      <c r="E96" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A96-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F96" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A96-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G96" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H96" s="75">
+        <f>100*(IF(INT((A96-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A96-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A96-1)/4)+1)-IF(INT((A96-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A96-1)/4))))*(MOD(A96-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>16.182107767497868</v>
+      </c>
+      <c r="I96" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A97" s="53">
+        <v>92</v>
+      </c>
+      <c r="B97" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>22:45</v>
+      </c>
+      <c r="C97" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>23:00</v>
+      </c>
+      <c r="D97" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A97-1)/4)+1)</f>
+        <v>6.2</v>
+      </c>
+      <c r="E97" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A97-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F97" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A97-1)/4)+1)</f>
+        <v>8</v>
+      </c>
+      <c r="G97" s="45">
+        <f t="shared" si="10"/>
+        <v>-8</v>
+      </c>
+      <c r="H97" s="75">
+        <f>100*(IF(INT((A97-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A97-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A97-1)/4)+1)-IF(INT((A97-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A97-1)/4))))*(MOD(A97-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>12.94568621399829</v>
+      </c>
+      <c r="I97" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A98" s="53">
+        <v>93</v>
+      </c>
+      <c r="B98" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>23:00</v>
+      </c>
+      <c r="C98" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>23:15</v>
+      </c>
+      <c r="D98" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A98-1)/4)+1)</f>
+        <v>5</v>
+      </c>
+      <c r="E98" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A98-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F98" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A98-1)/4)+1)</f>
+        <v>7.9999999999999849</v>
+      </c>
+      <c r="G98" s="45">
+        <f t="shared" si="10"/>
+        <v>-7.9999999999999849</v>
+      </c>
+      <c r="H98" s="75">
+        <f>100*(IF(INT((A98-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A98-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A98-1)/4)+1)-IF(INT((A98-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A98-1)/4))))*(MOD(A98-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>9.7092646604987181</v>
+      </c>
+      <c r="I98" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A99" s="53">
+        <v>94</v>
+      </c>
+      <c r="B99" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>23:15</v>
+      </c>
+      <c r="C99" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>23:30</v>
+      </c>
+      <c r="D99" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A99-1)/4)+1)</f>
+        <v>5</v>
+      </c>
+      <c r="E99" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A99-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F99" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A99-1)/4)+1)</f>
+        <v>7.9999999999999849</v>
+      </c>
+      <c r="G99" s="45">
+        <f t="shared" si="10"/>
+        <v>-7.9999999999999849</v>
+      </c>
+      <c r="H99" s="75">
+        <f>100*(IF(INT((A99-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A99-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A99-1)/4)+1)-IF(INT((A99-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A99-1)/4))))*(MOD(A99-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>6.4728431069991448</v>
+      </c>
+      <c r="I99" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A100" s="53">
+        <v>95</v>
+      </c>
+      <c r="B100" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>23:30</v>
+      </c>
+      <c r="C100" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>23:45</v>
+      </c>
+      <c r="D100" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A100-1)/4)+1)</f>
+        <v>5</v>
+      </c>
+      <c r="E100" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A100-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F100" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A100-1)/4)+1)</f>
+        <v>7.9999999999999849</v>
+      </c>
+      <c r="G100" s="45">
+        <f t="shared" si="10"/>
+        <v>-7.9999999999999849</v>
+      </c>
+      <c r="H100" s="75">
+        <f>100*(IF(INT((A100-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A100-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A100-1)/4)+1)-IF(INT((A100-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A100-1)/4))))*(MOD(A100-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>3.2364215534995715</v>
+      </c>
+      <c r="I100" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A101" s="53">
+        <v>96</v>
+      </c>
+      <c r="B101" s="42" t="str">
+        <f t="shared" si="8"/>
+        <v>23:45</v>
+      </c>
+      <c r="C101" s="42" t="str">
+        <f t="shared" si="9"/>
+        <v>24:00</v>
+      </c>
+      <c r="D101" s="52">
+        <f>INDEX('02_Dispatch'!$C$21:$C$44,INT((A101-1)/4)+1)</f>
+        <v>5</v>
+      </c>
+      <c r="E101" s="45">
+        <f>INDEX('02_Dispatch'!$H$21:$H$44,INT((A101-1)/4)+1)</f>
+        <v>0</v>
+      </c>
+      <c r="F101" s="45">
+        <f>INDEX('02_Dispatch'!$I$21:$I$44,INT((A101-1)/4)+1)</f>
+        <v>7.9999999999999849</v>
+      </c>
+      <c r="G101" s="45">
+        <f t="shared" si="10"/>
+        <v>-7.9999999999999849</v>
+      </c>
+      <c r="H101" s="75">
+        <f>100*(IF(INT((A101-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A101-1)/4)))+(INDEX('02_Dispatch'!$J$21:$J$44,INT((A101-1)/4)+1)-IF(INT((A101-1)/4)=0,0,INDEX('02_Dispatch'!$J$21:$J$44,INT((A101-1)/4))))*(MOD(A101-1,4)+1)/4)/'00_Inputs'!$B$14</f>
+        <v>0</v>
+      </c>
+      <c r="I101" s="42" t="str">
+        <f t="shared" si="11"/>
+        <v>DISCHARGE</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A103" s="3" t="s">
+        <v>221</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -5134,26 +8793,26 @@
         <v>96</v>
       </c>
       <c r="B1" s="40" t="s">
-        <v>211</v>
+        <v>222</v>
       </c>
       <c r="C1" s="40" t="s">
-        <v>212</v>
+        <v>223</v>
       </c>
       <c r="D1" s="40" t="s">
-        <v>213</v>
+        <v>224</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="41">
         <v>0</v>
       </c>
-      <c r="B2" s="75">
+      <c r="B2" s="76">
         <v>4.2</v>
       </c>
-      <c r="C2" s="75">
+      <c r="C2" s="76">
         <v>5</v>
       </c>
-      <c r="D2" s="75">
+      <c r="D2" s="76">
         <v>3.8</v>
       </c>
     </row>
@@ -5161,13 +8820,13 @@
       <c r="A3" s="41">
         <v>1</v>
       </c>
-      <c r="B3" s="75">
+      <c r="B3" s="76">
         <v>3.9</v>
       </c>
-      <c r="C3" s="75">
+      <c r="C3" s="76">
         <v>4.5999999999999996</v>
       </c>
-      <c r="D3" s="75">
+      <c r="D3" s="76">
         <v>3.6</v>
       </c>
     </row>
@@ -5175,13 +8834,13 @@
       <c r="A4" s="41">
         <v>2</v>
       </c>
-      <c r="B4" s="75">
+      <c r="B4" s="76">
         <v>3.7</v>
       </c>
-      <c r="C4" s="75">
+      <c r="C4" s="76">
         <v>4.4000000000000004</v>
       </c>
-      <c r="D4" s="75">
+      <c r="D4" s="76">
         <v>3.5</v>
       </c>
     </row>
@@ -5189,13 +8848,13 @@
       <c r="A5" s="41">
         <v>3</v>
       </c>
-      <c r="B5" s="75">
+      <c r="B5" s="76">
         <v>3.6</v>
       </c>
-      <c r="C5" s="75">
+      <c r="C5" s="76">
         <v>4.3</v>
       </c>
-      <c r="D5" s="75">
+      <c r="D5" s="76">
         <v>3.4</v>
       </c>
     </row>
@@ -5203,13 +8862,13 @@
       <c r="A6" s="41">
         <v>4</v>
       </c>
-      <c r="B6" s="75">
+      <c r="B6" s="76">
         <v>3.5</v>
       </c>
-      <c r="C6" s="75">
+      <c r="C6" s="76">
         <v>4.4000000000000004</v>
       </c>
-      <c r="D6" s="75">
+      <c r="D6" s="76">
         <v>3.4</v>
       </c>
     </row>
@@ -5217,13 +8876,13 @@
       <c r="A7" s="41">
         <v>5</v>
       </c>
-      <c r="B7" s="75">
+      <c r="B7" s="76">
         <v>3.8</v>
       </c>
-      <c r="C7" s="75">
+      <c r="C7" s="76">
         <v>4.8</v>
       </c>
-      <c r="D7" s="75">
+      <c r="D7" s="76">
         <v>3.6</v>
       </c>
     </row>
@@ -5231,13 +8890,13 @@
       <c r="A8" s="41">
         <v>6</v>
       </c>
-      <c r="B8" s="75">
+      <c r="B8" s="76">
         <v>4.5999999999999996</v>
       </c>
-      <c r="C8" s="75">
+      <c r="C8" s="76">
         <v>5.8</v>
       </c>
-      <c r="D8" s="75">
+      <c r="D8" s="76">
         <v>4</v>
       </c>
     </row>
@@ -5245,13 +8904,13 @@
       <c r="A9" s="41">
         <v>7</v>
       </c>
-      <c r="B9" s="75">
+      <c r="B9" s="76">
         <v>5.4</v>
       </c>
-      <c r="C9" s="75">
+      <c r="C9" s="76">
         <v>6.8</v>
       </c>
-      <c r="D9" s="75">
+      <c r="D9" s="76">
         <v>4.4000000000000004</v>
       </c>
     </row>
@@ -5259,13 +8918,13 @@
       <c r="A10" s="41">
         <v>8</v>
       </c>
-      <c r="B10" s="75">
+      <c r="B10" s="76">
         <v>5.2</v>
       </c>
-      <c r="C10" s="75">
+      <c r="C10" s="76">
         <v>6.2</v>
       </c>
-      <c r="D10" s="75">
+      <c r="D10" s="76">
         <v>4.4000000000000004</v>
       </c>
     </row>
@@ -5273,13 +8932,13 @@
       <c r="A11" s="41">
         <v>9</v>
       </c>
-      <c r="B11" s="75">
+      <c r="B11" s="76">
         <v>4</v>
       </c>
-      <c r="C11" s="75">
+      <c r="C11" s="76">
         <v>4.5999999999999996</v>
       </c>
-      <c r="D11" s="75">
+      <c r="D11" s="76">
         <v>4</v>
       </c>
     </row>
@@ -5287,13 +8946,13 @@
       <c r="A12" s="41">
         <v>10</v>
       </c>
-      <c r="B12" s="75">
+      <c r="B12" s="76">
         <v>3</v>
       </c>
-      <c r="C12" s="75">
+      <c r="C12" s="76">
         <v>3.2</v>
       </c>
-      <c r="D12" s="75">
+      <c r="D12" s="76">
         <v>3.7</v>
       </c>
     </row>
@@ -5301,13 +8960,13 @@
       <c r="A13" s="41">
         <v>11</v>
       </c>
-      <c r="B13" s="75">
+      <c r="B13" s="76">
         <v>2.6</v>
       </c>
-      <c r="C13" s="75">
+      <c r="C13" s="76">
         <v>2.6</v>
       </c>
-      <c r="D13" s="75">
+      <c r="D13" s="76">
         <v>3.5</v>
       </c>
     </row>
@@ -5315,13 +8974,13 @@
       <c r="A14" s="41">
         <v>12</v>
       </c>
-      <c r="B14" s="75">
+      <c r="B14" s="76">
         <v>2.4</v>
       </c>
-      <c r="C14" s="75">
+      <c r="C14" s="76">
         <v>2.2999999999999998</v>
       </c>
-      <c r="D14" s="75">
+      <c r="D14" s="76">
         <v>3.4</v>
       </c>
     </row>
@@ -5329,13 +8988,13 @@
       <c r="A15" s="41">
         <v>13</v>
       </c>
-      <c r="B15" s="75">
+      <c r="B15" s="76">
         <v>2.4</v>
       </c>
-      <c r="C15" s="75">
+      <c r="C15" s="76">
         <v>2.2000000000000002</v>
       </c>
-      <c r="D15" s="75">
+      <c r="D15" s="76">
         <v>3.4</v>
       </c>
     </row>
@@ -5343,13 +9002,13 @@
       <c r="A16" s="41">
         <v>14</v>
       </c>
-      <c r="B16" s="75">
+      <c r="B16" s="76">
         <v>2.6</v>
       </c>
-      <c r="C16" s="75">
+      <c r="C16" s="76">
         <v>2.5</v>
       </c>
-      <c r="D16" s="75">
+      <c r="D16" s="76">
         <v>3.5</v>
       </c>
     </row>
@@ -5357,13 +9016,13 @@
       <c r="A17" s="41">
         <v>15</v>
       </c>
-      <c r="B17" s="75">
+      <c r="B17" s="76">
         <v>3.1</v>
       </c>
-      <c r="C17" s="75">
+      <c r="C17" s="76">
         <v>3.4</v>
       </c>
-      <c r="D17" s="75">
+      <c r="D17" s="76">
         <v>3.7</v>
       </c>
     </row>
@@ -5371,13 +9030,13 @@
       <c r="A18" s="41">
         <v>16</v>
       </c>
-      <c r="B18" s="75">
+      <c r="B18" s="76">
         <v>4</v>
       </c>
-      <c r="C18" s="75">
+      <c r="C18" s="76">
         <v>5.2</v>
       </c>
-      <c r="D18" s="75">
+      <c r="D18" s="76">
         <v>4.0999999999999996</v>
       </c>
     </row>
@@ -5385,13 +9044,13 @@
       <c r="A19" s="41">
         <v>17</v>
       </c>
-      <c r="B19" s="75">
+      <c r="B19" s="76">
         <v>5.6</v>
       </c>
-      <c r="C19" s="75">
+      <c r="C19" s="76">
         <v>7.4</v>
       </c>
-      <c r="D19" s="75">
+      <c r="D19" s="76">
         <v>4.7</v>
       </c>
     </row>
@@ -5399,13 +9058,13 @@
       <c r="A20" s="41">
         <v>18</v>
       </c>
-      <c r="B20" s="75">
+      <c r="B20" s="76">
         <v>7.2</v>
       </c>
-      <c r="C20" s="75">
+      <c r="C20" s="76">
         <v>9.6</v>
       </c>
-      <c r="D20" s="75">
+      <c r="D20" s="76">
         <v>5.4</v>
       </c>
     </row>
@@ -5413,13 +9072,13 @@
       <c r="A21" s="41">
         <v>19</v>
       </c>
-      <c r="B21" s="75">
+      <c r="B21" s="76">
         <v>8.5</v>
       </c>
-      <c r="C21" s="75">
+      <c r="C21" s="76">
         <v>10</v>
       </c>
-      <c r="D21" s="75">
+      <c r="D21" s="76">
         <v>5.8</v>
       </c>
     </row>
@@ -5427,13 +9086,13 @@
       <c r="A22" s="41">
         <v>20</v>
       </c>
-      <c r="B22" s="75">
+      <c r="B22" s="76">
         <v>8.9</v>
       </c>
-      <c r="C22" s="75">
+      <c r="C22" s="76">
         <v>10</v>
       </c>
-      <c r="D22" s="75">
+      <c r="D22" s="76">
         <v>5.7</v>
       </c>
     </row>
@@ -5441,13 +9100,13 @@
       <c r="A23" s="41">
         <v>21</v>
       </c>
-      <c r="B23" s="75">
+      <c r="B23" s="76">
         <v>7.8</v>
       </c>
-      <c r="C23" s="75">
+      <c r="C23" s="76">
         <v>9.1999999999999993</v>
       </c>
-      <c r="D23" s="75">
+      <c r="D23" s="76">
         <v>5.2</v>
       </c>
     </row>
@@ -5455,13 +9114,13 @@
       <c r="A24" s="41">
         <v>22</v>
       </c>
-      <c r="B24" s="75">
+      <c r="B24" s="76">
         <v>6.2</v>
       </c>
-      <c r="C24" s="75">
+      <c r="C24" s="76">
         <v>7.4</v>
       </c>
-      <c r="D24" s="75">
+      <c r="D24" s="76">
         <v>4.5999999999999996</v>
       </c>
     </row>
@@ -5469,19 +9128,19 @@
       <c r="A25" s="41">
         <v>23</v>
       </c>
-      <c r="B25" s="75">
+      <c r="B25" s="76">
         <v>5</v>
       </c>
-      <c r="C25" s="75">
+      <c r="C25" s="76">
         <v>6</v>
       </c>
-      <c r="D25" s="75">
+      <c r="D25" s="76">
         <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>